<commit_message>
Reset Excel Table for CNC3X-06
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-06.xlsx
+++ b/FM-MN-07_CNC3X-06.xlsx
@@ -1804,17 +1804,9 @@
           <t>Worm up เครื่องจักร 15 นาที ทุกครั้งที่ใช้งาน</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C6" s="23" t="inlineStr"/>
       <c r="D6" s="22" t="inlineStr"/>
-      <c r="E6" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E6" s="23" t="inlineStr"/>
       <c r="F6" s="22" t="inlineStr"/>
       <c r="G6" s="22" t="inlineStr"/>
       <c r="H6" s="22" t="inlineStr"/>
@@ -1853,17 +1845,9 @@
           <t>เช็คระดับนำมันที่ Pump Hydraulic ทุกวัน เติมเมื่อพร่อง</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C7" s="23" t="inlineStr"/>
       <c r="D7" s="22" t="inlineStr"/>
-      <c r="E7" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E7" s="23" t="inlineStr"/>
       <c r="F7" s="22" t="inlineStr"/>
       <c r="G7" s="22" t="inlineStr"/>
       <c r="H7" s="22" t="inlineStr"/>
@@ -1902,17 +1886,9 @@
           <t>ทำความสะอาด Air filter Mesh ทุกวัน</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C8" s="23" t="inlineStr"/>
       <c r="D8" s="22" t="inlineStr"/>
-      <c r="E8" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E8" s="23" t="inlineStr"/>
       <c r="F8" s="22" t="inlineStr"/>
       <c r="G8" s="22" t="inlineStr"/>
       <c r="H8" s="22" t="inlineStr"/>
@@ -1951,17 +1927,9 @@
           <t>ตรวจเช็คแรงดัน Air Control Unit ปกติเฉลี่ยที่ 0.5 Mpa</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C9" s="23" t="inlineStr"/>
       <c r="D9" s="22" t="inlineStr"/>
-      <c r="E9" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E9" s="23" t="inlineStr"/>
       <c r="F9" s="22" t="inlineStr"/>
       <c r="G9" s="22" t="inlineStr"/>
       <c r="H9" s="22" t="inlineStr"/>
@@ -2000,17 +1968,9 @@
           <t>เช็คน้ำมันชุด Gear ของ ATC ทุกวัน(เปลี่ยนถ่ายทุกปี)</t>
         </is>
       </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C10" s="23" t="inlineStr"/>
       <c r="D10" s="22" t="inlineStr"/>
-      <c r="E10" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E10" s="23" t="inlineStr"/>
       <c r="F10" s="22" t="inlineStr"/>
       <c r="G10" s="22" t="inlineStr"/>
       <c r="H10" s="22" t="inlineStr"/>
@@ -2051,11 +2011,7 @@
       </c>
       <c r="C11" s="22" t="inlineStr"/>
       <c r="D11" s="22" t="inlineStr"/>
-      <c r="E11" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E11" s="23" t="inlineStr"/>
       <c r="F11" s="22" t="inlineStr"/>
       <c r="G11" s="22" t="inlineStr"/>
       <c r="H11" s="22" t="inlineStr"/>
@@ -2094,17 +2050,9 @@
           <t>ตรวจสอบการเคลื่อนที่ของแกนทุกแกน (X,Y,Z)</t>
         </is>
       </c>
-      <c r="C12" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C12" s="23" t="inlineStr"/>
       <c r="D12" s="22" t="inlineStr"/>
-      <c r="E12" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E12" s="23" t="inlineStr"/>
       <c r="F12" s="22" t="inlineStr"/>
       <c r="G12" s="22" t="inlineStr"/>
       <c r="H12" s="22" t="inlineStr"/>
@@ -2145,11 +2093,7 @@
       </c>
       <c r="C13" s="22" t="inlineStr"/>
       <c r="D13" s="22" t="inlineStr"/>
-      <c r="E13" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E13" s="23" t="inlineStr"/>
       <c r="F13" s="22" t="inlineStr"/>
       <c r="G13" s="22" t="inlineStr"/>
       <c r="H13" s="22" t="inlineStr"/>
@@ -2188,17 +2132,9 @@
           <t>การทำงานของ Coolant pump</t>
         </is>
       </c>
-      <c r="C14" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C14" s="23" t="inlineStr"/>
       <c r="D14" s="22" t="inlineStr"/>
-      <c r="E14" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E14" s="23" t="inlineStr"/>
       <c r="F14" s="22" t="inlineStr"/>
       <c r="G14" s="22" t="inlineStr"/>
       <c r="H14" s="22" t="inlineStr"/>
@@ -2239,11 +2175,7 @@
       </c>
       <c r="C15" s="22" t="inlineStr"/>
       <c r="D15" s="22" t="inlineStr"/>
-      <c r="E15" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E15" s="23" t="inlineStr"/>
       <c r="F15" s="22" t="inlineStr"/>
       <c r="G15" s="22" t="inlineStr"/>
       <c r="H15" s="22" t="inlineStr"/>
@@ -2284,11 +2216,7 @@
       </c>
       <c r="C16" s="22" t="inlineStr"/>
       <c r="D16" s="22" t="inlineStr"/>
-      <c r="E16" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E16" s="23" t="inlineStr"/>
       <c r="F16" s="22" t="inlineStr"/>
       <c r="G16" s="22" t="inlineStr"/>
       <c r="H16" s="22" t="inlineStr"/>
@@ -2327,17 +2255,9 @@
           <t>การทำงานของ Arm เปลี่ยน Tool</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C17" s="23" t="inlineStr"/>
       <c r="D17" s="22" t="inlineStr"/>
-      <c r="E17" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E17" s="23" t="inlineStr"/>
       <c r="F17" s="22" t="inlineStr"/>
       <c r="G17" s="22" t="inlineStr"/>
       <c r="H17" s="22" t="inlineStr"/>
@@ -2376,17 +2296,9 @@
           <t>ตรวจสอบระดับของน้ำ Coolant เติมเมื่ออยู่ระดับที่ต่ำ</t>
         </is>
       </c>
-      <c r="C18" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C18" s="23" t="inlineStr"/>
       <c r="D18" s="22" t="inlineStr"/>
-      <c r="E18" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E18" s="23" t="inlineStr"/>
       <c r="F18" s="22" t="inlineStr"/>
       <c r="G18" s="22" t="inlineStr"/>
       <c r="H18" s="22" t="inlineStr"/>
@@ -2425,17 +2337,9 @@
           <t>ความสะอาดทั่วไปของเครื่องจักรโดยรวม</t>
         </is>
       </c>
-      <c r="C19" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C19" s="23" t="inlineStr"/>
       <c r="D19" s="22" t="inlineStr"/>
-      <c r="E19" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E19" s="23" t="inlineStr"/>
       <c r="F19" s="22" t="inlineStr"/>
       <c r="G19" s="22" t="inlineStr"/>
       <c r="H19" s="22" t="inlineStr"/>
@@ -2474,17 +2378,9 @@
           <t>ตรวจสอบความพร้อมสภาพโดยรวม(ฟังด้วยหู ดูด้วยตา)</t>
         </is>
       </c>
-      <c r="C20" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C20" s="23" t="inlineStr"/>
       <c r="D20" s="22" t="inlineStr"/>
-      <c r="E20" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E20" s="23" t="inlineStr"/>
       <c r="F20" s="22" t="inlineStr"/>
       <c r="G20" s="22" t="inlineStr"/>
       <c r="H20" s="22" t="inlineStr"/>
@@ -2523,17 +2419,9 @@
           <t>ตรวจสอบสายไฮโดรลิกส์ และสายลม</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C21" s="23" t="inlineStr"/>
       <c r="D21" s="22" t="inlineStr"/>
-      <c r="E21" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E21" s="23" t="inlineStr"/>
       <c r="F21" s="22" t="inlineStr"/>
       <c r="G21" s="22" t="inlineStr"/>
       <c r="H21" s="22" t="inlineStr"/>
@@ -2566,17 +2454,9 @@
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="3" t="n"/>
       <c r="B22" s="8" t="n"/>
-      <c r="C22" s="33" t="inlineStr">
-        <is>
-          <t>ณัช วิกรัยเจริญ</t>
-        </is>
-      </c>
+      <c r="C22" s="33" t="inlineStr"/>
       <c r="D22" s="28" t="inlineStr"/>
-      <c r="E22" s="33" t="inlineStr">
-        <is>
-          <t>ณัช วิกรัยเจริญ</t>
-        </is>
-      </c>
+      <c r="E22" s="33" t="inlineStr"/>
       <c r="F22" s="28" t="inlineStr"/>
       <c r="G22" s="28" t="inlineStr"/>
       <c r="H22" s="28" t="inlineStr"/>

</xml_diff>

<commit_message>
Direct Write Excel for CNC3X-06 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-06.xlsx
+++ b/FM-MN-07_CNC3X-06.xlsx
@@ -1809,7 +1809,11 @@
       <c r="E6" s="23" t="inlineStr"/>
       <c r="F6" s="22" t="inlineStr"/>
       <c r="G6" s="22" t="inlineStr"/>
-      <c r="H6" s="22" t="inlineStr"/>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="22" t="inlineStr"/>
       <c r="J6" s="22" t="inlineStr"/>
       <c r="K6" s="22" t="inlineStr"/>
@@ -1850,7 +1854,11 @@
       <c r="E7" s="23" t="inlineStr"/>
       <c r="F7" s="22" t="inlineStr"/>
       <c r="G7" s="22" t="inlineStr"/>
-      <c r="H7" s="22" t="inlineStr"/>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="22" t="inlineStr"/>
       <c r="J7" s="22" t="inlineStr"/>
       <c r="K7" s="22" t="inlineStr"/>
@@ -1891,7 +1899,11 @@
       <c r="E8" s="23" t="inlineStr"/>
       <c r="F8" s="22" t="inlineStr"/>
       <c r="G8" s="22" t="inlineStr"/>
-      <c r="H8" s="22" t="inlineStr"/>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="22" t="inlineStr"/>
       <c r="J8" s="22" t="inlineStr"/>
       <c r="K8" s="22" t="inlineStr"/>
@@ -1932,7 +1944,11 @@
       <c r="E9" s="23" t="inlineStr"/>
       <c r="F9" s="22" t="inlineStr"/>
       <c r="G9" s="22" t="inlineStr"/>
-      <c r="H9" s="22" t="inlineStr"/>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="22" t="inlineStr"/>
       <c r="J9" s="22" t="inlineStr"/>
       <c r="K9" s="22" t="inlineStr"/>
@@ -1973,7 +1989,11 @@
       <c r="E10" s="23" t="inlineStr"/>
       <c r="F10" s="22" t="inlineStr"/>
       <c r="G10" s="22" t="inlineStr"/>
-      <c r="H10" s="22" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="22" t="inlineStr"/>
       <c r="J10" s="22" t="inlineStr"/>
       <c r="K10" s="22" t="inlineStr"/>
@@ -2014,7 +2034,11 @@
       <c r="E11" s="23" t="inlineStr"/>
       <c r="F11" s="22" t="inlineStr"/>
       <c r="G11" s="22" t="inlineStr"/>
-      <c r="H11" s="22" t="inlineStr"/>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I11" s="22" t="inlineStr"/>
       <c r="J11" s="22" t="inlineStr"/>
       <c r="K11" s="22" t="inlineStr"/>
@@ -2055,7 +2079,11 @@
       <c r="E12" s="23" t="inlineStr"/>
       <c r="F12" s="22" t="inlineStr"/>
       <c r="G12" s="22" t="inlineStr"/>
-      <c r="H12" s="22" t="inlineStr"/>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I12" s="22" t="inlineStr"/>
       <c r="J12" s="22" t="inlineStr"/>
       <c r="K12" s="22" t="inlineStr"/>
@@ -2096,7 +2124,11 @@
       <c r="E13" s="23" t="inlineStr"/>
       <c r="F13" s="22" t="inlineStr"/>
       <c r="G13" s="22" t="inlineStr"/>
-      <c r="H13" s="22" t="inlineStr"/>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I13" s="22" t="inlineStr"/>
       <c r="J13" s="22" t="inlineStr"/>
       <c r="K13" s="22" t="inlineStr"/>
@@ -2137,7 +2169,11 @@
       <c r="E14" s="23" t="inlineStr"/>
       <c r="F14" s="22" t="inlineStr"/>
       <c r="G14" s="22" t="inlineStr"/>
-      <c r="H14" s="22" t="inlineStr"/>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I14" s="22" t="inlineStr"/>
       <c r="J14" s="22" t="inlineStr"/>
       <c r="K14" s="22" t="inlineStr"/>
@@ -2178,7 +2214,11 @@
       <c r="E15" s="23" t="inlineStr"/>
       <c r="F15" s="22" t="inlineStr"/>
       <c r="G15" s="22" t="inlineStr"/>
-      <c r="H15" s="22" t="inlineStr"/>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I15" s="22" t="inlineStr"/>
       <c r="J15" s="22" t="inlineStr"/>
       <c r="K15" s="22" t="inlineStr"/>
@@ -2219,7 +2259,11 @@
       <c r="E16" s="23" t="inlineStr"/>
       <c r="F16" s="22" t="inlineStr"/>
       <c r="G16" s="22" t="inlineStr"/>
-      <c r="H16" s="22" t="inlineStr"/>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I16" s="22" t="inlineStr"/>
       <c r="J16" s="22" t="inlineStr"/>
       <c r="K16" s="22" t="inlineStr"/>
@@ -2260,7 +2304,11 @@
       <c r="E17" s="23" t="inlineStr"/>
       <c r="F17" s="22" t="inlineStr"/>
       <c r="G17" s="22" t="inlineStr"/>
-      <c r="H17" s="22" t="inlineStr"/>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I17" s="22" t="inlineStr"/>
       <c r="J17" s="22" t="inlineStr"/>
       <c r="K17" s="22" t="inlineStr"/>
@@ -2301,7 +2349,11 @@
       <c r="E18" s="23" t="inlineStr"/>
       <c r="F18" s="22" t="inlineStr"/>
       <c r="G18" s="22" t="inlineStr"/>
-      <c r="H18" s="22" t="inlineStr"/>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I18" s="22" t="inlineStr"/>
       <c r="J18" s="22" t="inlineStr"/>
       <c r="K18" s="22" t="inlineStr"/>
@@ -2342,7 +2394,11 @@
       <c r="E19" s="23" t="inlineStr"/>
       <c r="F19" s="22" t="inlineStr"/>
       <c r="G19" s="22" t="inlineStr"/>
-      <c r="H19" s="22" t="inlineStr"/>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I19" s="22" t="inlineStr"/>
       <c r="J19" s="22" t="inlineStr"/>
       <c r="K19" s="22" t="inlineStr"/>
@@ -2383,7 +2439,11 @@
       <c r="E20" s="23" t="inlineStr"/>
       <c r="F20" s="22" t="inlineStr"/>
       <c r="G20" s="22" t="inlineStr"/>
-      <c r="H20" s="22" t="inlineStr"/>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I20" s="22" t="inlineStr"/>
       <c r="J20" s="22" t="inlineStr"/>
       <c r="K20" s="22" t="inlineStr"/>
@@ -2424,7 +2484,11 @@
       <c r="E21" s="23" t="inlineStr"/>
       <c r="F21" s="22" t="inlineStr"/>
       <c r="G21" s="22" t="inlineStr"/>
-      <c r="H21" s="22" t="inlineStr"/>
+      <c r="H21" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I21" s="22" t="inlineStr"/>
       <c r="J21" s="22" t="inlineStr"/>
       <c r="K21" s="22" t="inlineStr"/>
@@ -2459,7 +2523,11 @@
       <c r="E22" s="33" t="inlineStr"/>
       <c r="F22" s="28" t="inlineStr"/>
       <c r="G22" s="28" t="inlineStr"/>
-      <c r="H22" s="28" t="inlineStr"/>
+      <c r="H22" s="33" t="inlineStr">
+        <is>
+          <t>นาย ภูริทัศน์ ปิ่นโต</t>
+        </is>
+      </c>
       <c r="I22" s="28" t="inlineStr"/>
       <c r="J22" s="28" t="inlineStr"/>
       <c r="K22" s="28" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CNC3X-06 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-06.xlsx
+++ b/FM-MN-07_CNC3X-06.xlsx
@@ -1815,7 +1815,11 @@
         </is>
       </c>
       <c r="I6" s="22" t="inlineStr"/>
-      <c r="J6" s="22" t="inlineStr"/>
+      <c r="J6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="22" t="inlineStr"/>
       <c r="L6" s="22" t="inlineStr"/>
       <c r="M6" s="22" t="inlineStr"/>
@@ -1860,7 +1864,11 @@
         </is>
       </c>
       <c r="I7" s="22" t="inlineStr"/>
-      <c r="J7" s="22" t="inlineStr"/>
+      <c r="J7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="22" t="inlineStr"/>
       <c r="L7" s="22" t="inlineStr"/>
       <c r="M7" s="22" t="inlineStr"/>
@@ -1905,7 +1913,11 @@
         </is>
       </c>
       <c r="I8" s="22" t="inlineStr"/>
-      <c r="J8" s="22" t="inlineStr"/>
+      <c r="J8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="22" t="inlineStr"/>
       <c r="L8" s="22" t="inlineStr"/>
       <c r="M8" s="22" t="inlineStr"/>
@@ -1950,7 +1962,11 @@
         </is>
       </c>
       <c r="I9" s="22" t="inlineStr"/>
-      <c r="J9" s="22" t="inlineStr"/>
+      <c r="J9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="22" t="inlineStr"/>
       <c r="L9" s="22" t="inlineStr"/>
       <c r="M9" s="22" t="inlineStr"/>
@@ -1995,7 +2011,11 @@
         </is>
       </c>
       <c r="I10" s="22" t="inlineStr"/>
-      <c r="J10" s="22" t="inlineStr"/>
+      <c r="J10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="22" t="inlineStr"/>
       <c r="L10" s="22" t="inlineStr"/>
       <c r="M10" s="22" t="inlineStr"/>
@@ -2040,7 +2060,11 @@
         </is>
       </c>
       <c r="I11" s="22" t="inlineStr"/>
-      <c r="J11" s="22" t="inlineStr"/>
+      <c r="J11" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K11" s="22" t="inlineStr"/>
       <c r="L11" s="22" t="inlineStr"/>
       <c r="M11" s="22" t="inlineStr"/>
@@ -2085,7 +2109,11 @@
         </is>
       </c>
       <c r="I12" s="22" t="inlineStr"/>
-      <c r="J12" s="22" t="inlineStr"/>
+      <c r="J12" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K12" s="22" t="inlineStr"/>
       <c r="L12" s="22" t="inlineStr"/>
       <c r="M12" s="22" t="inlineStr"/>
@@ -2130,7 +2158,11 @@
         </is>
       </c>
       <c r="I13" s="22" t="inlineStr"/>
-      <c r="J13" s="22" t="inlineStr"/>
+      <c r="J13" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K13" s="22" t="inlineStr"/>
       <c r="L13" s="22" t="inlineStr"/>
       <c r="M13" s="22" t="inlineStr"/>
@@ -2175,7 +2207,11 @@
         </is>
       </c>
       <c r="I14" s="22" t="inlineStr"/>
-      <c r="J14" s="22" t="inlineStr"/>
+      <c r="J14" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K14" s="22" t="inlineStr"/>
       <c r="L14" s="22" t="inlineStr"/>
       <c r="M14" s="22" t="inlineStr"/>
@@ -2220,7 +2256,11 @@
         </is>
       </c>
       <c r="I15" s="22" t="inlineStr"/>
-      <c r="J15" s="22" t="inlineStr"/>
+      <c r="J15" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K15" s="22" t="inlineStr"/>
       <c r="L15" s="22" t="inlineStr"/>
       <c r="M15" s="22" t="inlineStr"/>
@@ -2265,7 +2305,11 @@
         </is>
       </c>
       <c r="I16" s="22" t="inlineStr"/>
-      <c r="J16" s="22" t="inlineStr"/>
+      <c r="J16" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K16" s="22" t="inlineStr"/>
       <c r="L16" s="22" t="inlineStr"/>
       <c r="M16" s="22" t="inlineStr"/>
@@ -2310,7 +2354,11 @@
         </is>
       </c>
       <c r="I17" s="22" t="inlineStr"/>
-      <c r="J17" s="22" t="inlineStr"/>
+      <c r="J17" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K17" s="22" t="inlineStr"/>
       <c r="L17" s="22" t="inlineStr"/>
       <c r="M17" s="22" t="inlineStr"/>
@@ -2355,7 +2403,11 @@
         </is>
       </c>
       <c r="I18" s="22" t="inlineStr"/>
-      <c r="J18" s="22" t="inlineStr"/>
+      <c r="J18" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K18" s="22" t="inlineStr"/>
       <c r="L18" s="22" t="inlineStr"/>
       <c r="M18" s="22" t="inlineStr"/>
@@ -2400,7 +2452,11 @@
         </is>
       </c>
       <c r="I19" s="22" t="inlineStr"/>
-      <c r="J19" s="22" t="inlineStr"/>
+      <c r="J19" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K19" s="22" t="inlineStr"/>
       <c r="L19" s="22" t="inlineStr"/>
       <c r="M19" s="22" t="inlineStr"/>
@@ -2445,7 +2501,11 @@
         </is>
       </c>
       <c r="I20" s="22" t="inlineStr"/>
-      <c r="J20" s="22" t="inlineStr"/>
+      <c r="J20" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K20" s="22" t="inlineStr"/>
       <c r="L20" s="22" t="inlineStr"/>
       <c r="M20" s="22" t="inlineStr"/>
@@ -2490,7 +2550,11 @@
         </is>
       </c>
       <c r="I21" s="22" t="inlineStr"/>
-      <c r="J21" s="22" t="inlineStr"/>
+      <c r="J21" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K21" s="22" t="inlineStr"/>
       <c r="L21" s="22" t="inlineStr"/>
       <c r="M21" s="22" t="inlineStr"/>
@@ -2529,7 +2593,11 @@
         </is>
       </c>
       <c r="I22" s="28" t="inlineStr"/>
-      <c r="J22" s="28" t="inlineStr"/>
+      <c r="J22" s="33" t="inlineStr">
+        <is>
+          <t>นาย ภูริทัศน์ ปิ่นโต</t>
+        </is>
+      </c>
       <c r="K22" s="28" t="inlineStr"/>
       <c r="L22" s="28" t="inlineStr"/>
       <c r="M22" s="28" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CNC3X-06 Day 9
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-06.xlsx
+++ b/FM-MN-07_CNC3X-06.xlsx
@@ -1820,7 +1820,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K6" s="22" t="inlineStr"/>
+      <c r="K6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L6" s="22" t="inlineStr"/>
       <c r="M6" s="22" t="inlineStr"/>
       <c r="N6" s="22" t="inlineStr"/>
@@ -1869,7 +1873,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K7" s="22" t="inlineStr"/>
+      <c r="K7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L7" s="22" t="inlineStr"/>
       <c r="M7" s="22" t="inlineStr"/>
       <c r="N7" s="22" t="inlineStr"/>
@@ -1918,7 +1926,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K8" s="22" t="inlineStr"/>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L8" s="22" t="inlineStr"/>
       <c r="M8" s="22" t="inlineStr"/>
       <c r="N8" s="22" t="inlineStr"/>
@@ -1967,7 +1979,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K9" s="22" t="inlineStr"/>
+      <c r="K9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L9" s="22" t="inlineStr"/>
       <c r="M9" s="22" t="inlineStr"/>
       <c r="N9" s="22" t="inlineStr"/>
@@ -2016,7 +2032,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K10" s="22" t="inlineStr"/>
+      <c r="K10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L10" s="22" t="inlineStr"/>
       <c r="M10" s="22" t="inlineStr"/>
       <c r="N10" s="22" t="inlineStr"/>
@@ -2065,7 +2085,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K11" s="22" t="inlineStr"/>
+      <c r="K11" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L11" s="22" t="inlineStr"/>
       <c r="M11" s="22" t="inlineStr"/>
       <c r="N11" s="22" t="inlineStr"/>
@@ -2114,7 +2138,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K12" s="22" t="inlineStr"/>
+      <c r="K12" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L12" s="22" t="inlineStr"/>
       <c r="M12" s="22" t="inlineStr"/>
       <c r="N12" s="22" t="inlineStr"/>
@@ -2163,7 +2191,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K13" s="22" t="inlineStr"/>
+      <c r="K13" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L13" s="22" t="inlineStr"/>
       <c r="M13" s="22" t="inlineStr"/>
       <c r="N13" s="22" t="inlineStr"/>
@@ -2212,7 +2244,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K14" s="22" t="inlineStr"/>
+      <c r="K14" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L14" s="22" t="inlineStr"/>
       <c r="M14" s="22" t="inlineStr"/>
       <c r="N14" s="22" t="inlineStr"/>
@@ -2261,7 +2297,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K15" s="22" t="inlineStr"/>
+      <c r="K15" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L15" s="22" t="inlineStr"/>
       <c r="M15" s="22" t="inlineStr"/>
       <c r="N15" s="22" t="inlineStr"/>
@@ -2310,7 +2350,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K16" s="22" t="inlineStr"/>
+      <c r="K16" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L16" s="22" t="inlineStr"/>
       <c r="M16" s="22" t="inlineStr"/>
       <c r="N16" s="22" t="inlineStr"/>
@@ -2359,7 +2403,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K17" s="22" t="inlineStr"/>
+      <c r="K17" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L17" s="22" t="inlineStr"/>
       <c r="M17" s="22" t="inlineStr"/>
       <c r="N17" s="22" t="inlineStr"/>
@@ -2408,7 +2456,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K18" s="22" t="inlineStr"/>
+      <c r="K18" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L18" s="22" t="inlineStr"/>
       <c r="M18" s="22" t="inlineStr"/>
       <c r="N18" s="22" t="inlineStr"/>
@@ -2457,7 +2509,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K19" s="22" t="inlineStr"/>
+      <c r="K19" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L19" s="22" t="inlineStr"/>
       <c r="M19" s="22" t="inlineStr"/>
       <c r="N19" s="22" t="inlineStr"/>
@@ -2506,7 +2562,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K20" s="22" t="inlineStr"/>
+      <c r="K20" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L20" s="22" t="inlineStr"/>
       <c r="M20" s="22" t="inlineStr"/>
       <c r="N20" s="22" t="inlineStr"/>
@@ -2555,7 +2615,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K21" s="22" t="inlineStr"/>
+      <c r="K21" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L21" s="22" t="inlineStr"/>
       <c r="M21" s="22" t="inlineStr"/>
       <c r="N21" s="22" t="inlineStr"/>
@@ -2598,7 +2662,11 @@
           <t>นาย ภูริทัศน์ ปิ่นโต</t>
         </is>
       </c>
-      <c r="K22" s="28" t="inlineStr"/>
+      <c r="K22" s="33" t="inlineStr">
+        <is>
+          <t>นาย ภูริทัศน์ ปิ่นโต</t>
+        </is>
+      </c>
       <c r="L22" s="28" t="inlineStr"/>
       <c r="M22" s="28" t="inlineStr"/>
       <c r="N22" s="28" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CNC3X-06 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-06.xlsx
+++ b/FM-MN-07_CNC3X-06.xlsx
@@ -1825,7 +1825,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L6" s="22" t="inlineStr"/>
+      <c r="L6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="22" t="inlineStr"/>
       <c r="N6" s="22" t="inlineStr"/>
       <c r="O6" s="22" t="inlineStr"/>
@@ -1878,7 +1882,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L7" s="22" t="inlineStr"/>
+      <c r="L7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="22" t="inlineStr"/>
       <c r="N7" s="22" t="inlineStr"/>
       <c r="O7" s="22" t="inlineStr"/>
@@ -1931,7 +1939,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L8" s="22" t="inlineStr"/>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="22" t="inlineStr"/>
       <c r="N8" s="22" t="inlineStr"/>
       <c r="O8" s="22" t="inlineStr"/>
@@ -1984,7 +1996,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L9" s="22" t="inlineStr"/>
+      <c r="L9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="22" t="inlineStr"/>
       <c r="N9" s="22" t="inlineStr"/>
       <c r="O9" s="22" t="inlineStr"/>
@@ -2037,7 +2053,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L10" s="22" t="inlineStr"/>
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="22" t="inlineStr"/>
       <c r="N10" s="22" t="inlineStr"/>
       <c r="O10" s="22" t="inlineStr"/>
@@ -2090,7 +2110,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L11" s="22" t="inlineStr"/>
+      <c r="L11" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M11" s="22" t="inlineStr"/>
       <c r="N11" s="22" t="inlineStr"/>
       <c r="O11" s="22" t="inlineStr"/>
@@ -2143,7 +2167,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L12" s="22" t="inlineStr"/>
+      <c r="L12" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M12" s="22" t="inlineStr"/>
       <c r="N12" s="22" t="inlineStr"/>
       <c r="O12" s="22" t="inlineStr"/>
@@ -2196,7 +2224,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L13" s="22" t="inlineStr"/>
+      <c r="L13" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M13" s="22" t="inlineStr"/>
       <c r="N13" s="22" t="inlineStr"/>
       <c r="O13" s="22" t="inlineStr"/>
@@ -2249,7 +2281,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L14" s="22" t="inlineStr"/>
+      <c r="L14" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M14" s="22" t="inlineStr"/>
       <c r="N14" s="22" t="inlineStr"/>
       <c r="O14" s="22" t="inlineStr"/>
@@ -2302,7 +2338,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L15" s="22" t="inlineStr"/>
+      <c r="L15" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M15" s="22" t="inlineStr"/>
       <c r="N15" s="22" t="inlineStr"/>
       <c r="O15" s="22" t="inlineStr"/>
@@ -2355,7 +2395,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L16" s="22" t="inlineStr"/>
+      <c r="L16" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M16" s="22" t="inlineStr"/>
       <c r="N16" s="22" t="inlineStr"/>
       <c r="O16" s="22" t="inlineStr"/>
@@ -2408,7 +2452,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L17" s="22" t="inlineStr"/>
+      <c r="L17" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M17" s="22" t="inlineStr"/>
       <c r="N17" s="22" t="inlineStr"/>
       <c r="O17" s="22" t="inlineStr"/>
@@ -2461,7 +2509,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L18" s="22" t="inlineStr"/>
+      <c r="L18" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M18" s="22" t="inlineStr"/>
       <c r="N18" s="22" t="inlineStr"/>
       <c r="O18" s="22" t="inlineStr"/>
@@ -2514,7 +2566,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L19" s="22" t="inlineStr"/>
+      <c r="L19" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M19" s="22" t="inlineStr"/>
       <c r="N19" s="22" t="inlineStr"/>
       <c r="O19" s="22" t="inlineStr"/>
@@ -2567,7 +2623,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L20" s="22" t="inlineStr"/>
+      <c r="L20" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M20" s="22" t="inlineStr"/>
       <c r="N20" s="22" t="inlineStr"/>
       <c r="O20" s="22" t="inlineStr"/>
@@ -2620,7 +2680,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L21" s="22" t="inlineStr"/>
+      <c r="L21" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M21" s="22" t="inlineStr"/>
       <c r="N21" s="22" t="inlineStr"/>
       <c r="O21" s="22" t="inlineStr"/>
@@ -2667,7 +2731,11 @@
           <t>นาย ภูริทัศน์ ปิ่นโต</t>
         </is>
       </c>
-      <c r="L22" s="28" t="inlineStr"/>
+      <c r="L22" s="33" t="inlineStr">
+        <is>
+          <t>ภูริทัศน์ ปิ่นโต</t>
+        </is>
+      </c>
       <c r="M22" s="28" t="inlineStr"/>
       <c r="N22" s="28" t="inlineStr"/>
       <c r="O22" s="28" t="inlineStr"/>

</xml_diff>